<commit_message>
Novetats CIMA: 50 nous farmacos pendents de validacio
</commit_message>
<xml_diff>
--- a/inhaladors_MPOC_ASMA_Avanzado_FINAL.xlsx
+++ b/inhaladors_MPOC_ASMA_Avanzado_FINAL.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inhaladors MPOC ASMA" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Llegenda i instruccions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Inhaladors MPOC ASMA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Llegenda i instruccions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inhaladors MPOC ASMA'!$A$1:$P$97</definedName>
@@ -63,7 +63,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -95,6 +95,16 @@
         <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -116,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -144,6 +154,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -509,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P97"/>
+  <dimension ref="A1:P147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7022,6 +7038,3710 @@
         </is>
       </c>
     </row>
+    <row r="98" ht="40" customHeight="1">
+      <c r="A98" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B98" s="11" t="inlineStr">
+        <is>
+          <t>ACETILSALICILICO ACIDO</t>
+        </is>
+      </c>
+      <c r="C98" s="11" t="inlineStr">
+        <is>
+          <t>A.A.S. 100 mg COMPRIMIDOS, 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="inlineStr">
+        <is>
+          <t>686580</t>
+        </is>
+      </c>
+      <c r="E98" s="11" t="inlineStr">
+        <is>
+          <t>A.A.S. 100 mg COMPRIMIDOS, 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="F98" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G98" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H98" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I98" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J98" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K98" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L98" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M98" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=42991</t>
+        </is>
+      </c>
+      <c r="N98" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O98" s="11" t="inlineStr"/>
+      <c r="P98" s="11" t="inlineStr"/>
+    </row>
+    <row r="99" ht="40" customHeight="1">
+      <c r="A99" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B99" s="11" t="inlineStr">
+        <is>
+          <t>ACETILSALICILICO ACIDO</t>
+        </is>
+      </c>
+      <c r="C99" s="11" t="inlineStr">
+        <is>
+          <t>A.A.S. 500 mg COMPRIMIDOS , 20 comprimidos</t>
+        </is>
+      </c>
+      <c r="D99" s="11" t="inlineStr">
+        <is>
+          <t>700693</t>
+        </is>
+      </c>
+      <c r="E99" s="11" t="inlineStr">
+        <is>
+          <t>A.A.S. 500 mg COMPRIMIDOS , 20 comprimidos</t>
+        </is>
+      </c>
+      <c r="F99" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G99" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H99" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I99" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J99" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K99" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L99" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M99" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=42956</t>
+        </is>
+      </c>
+      <c r="N99" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O99" s="11" t="inlineStr"/>
+      <c r="P99" s="11" t="inlineStr"/>
+    </row>
+    <row r="100" ht="40" customHeight="1">
+      <c r="A100" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
+          <t>PARACETAMOL, FENILEFRINA BITARTRATO, CLORFENAMINA MALEATO</t>
+        </is>
+      </c>
+      <c r="C100" s="11" t="inlineStr">
+        <is>
+          <t>ABACAT GRANULADO PARA SOLUCIÓN ORAL. 10 sobres</t>
+        </is>
+      </c>
+      <c r="D100" s="11" t="inlineStr">
+        <is>
+          <t>692223</t>
+        </is>
+      </c>
+      <c r="E100" s="11" t="inlineStr">
+        <is>
+          <t>ABACAT GRANULADO PARA SOLUCIÓN ORAL. 10 sobres</t>
+        </is>
+      </c>
+      <c r="F100" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G100" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H100" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I100" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J100" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K100" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L100" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M100" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=76206</t>
+        </is>
+      </c>
+      <c r="N100" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O100" s="11" t="inlineStr"/>
+      <c r="P100" s="11" t="inlineStr"/>
+    </row>
+    <row r="101" ht="40" customHeight="1">
+      <c r="A101" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR</t>
+        </is>
+      </c>
+      <c r="C101" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR TARBIS 300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG 60 comprimidos (Blister Al/Al)</t>
+        </is>
+      </c>
+      <c r="D101" s="11" t="inlineStr">
+        <is>
+          <t>727637</t>
+        </is>
+      </c>
+      <c r="E101" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR TARBIS 300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG 60 comprimidos (Blister Al/Al)</t>
+        </is>
+      </c>
+      <c r="F101" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G101" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H101" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I101" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J101" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K101" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L101" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M101" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=84740</t>
+        </is>
+      </c>
+      <c r="N101" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O101" s="11" t="inlineStr"/>
+      <c r="P101" s="11" t="inlineStr"/>
+    </row>
+    <row r="102" ht="40" customHeight="1">
+      <c r="A102" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B102" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR, LAMIVUDINA</t>
+        </is>
+      </c>
+      <c r="C102" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA  DR. REDDYS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="D102" s="11" t="inlineStr">
+        <is>
+          <t>711415</t>
+        </is>
+      </c>
+      <c r="E102" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA  DR. REDDYS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="F102" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G102" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H102" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I102" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J102" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K102" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L102" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M102" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=81012</t>
+        </is>
+      </c>
+      <c r="N102" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O102" s="11" t="inlineStr"/>
+      <c r="P102" s="11" t="inlineStr"/>
+    </row>
+    <row r="103" ht="40" customHeight="1">
+      <c r="A103" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B103" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR SULFATO, LAMIVUDINA</t>
+        </is>
+      </c>
+      <c r="C103" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA AUROVITAS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="D103" s="11" t="inlineStr">
+        <is>
+          <t>715527</t>
+        </is>
+      </c>
+      <c r="E103" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA AUROVITAS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="F103" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G103" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H103" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I103" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J103" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K103" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L103" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M103" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=81926</t>
+        </is>
+      </c>
+      <c r="N103" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O103" s="11" t="inlineStr"/>
+      <c r="P103" s="11" t="inlineStr"/>
+    </row>
+    <row r="104" ht="40" customHeight="1">
+      <c r="A104" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B104" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR CLORHIDRATO, LAMIVUDINA</t>
+        </is>
+      </c>
+      <c r="C104" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA GLENMARK 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 30 comprimidos (Blister PVD/PVDC/Al)</t>
+        </is>
+      </c>
+      <c r="D104" s="11" t="inlineStr">
+        <is>
+          <t>719707</t>
+        </is>
+      </c>
+      <c r="E104" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA GLENMARK 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 30 comprimidos (Blister PVD/PVDC/Al)</t>
+        </is>
+      </c>
+      <c r="F104" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G104" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H104" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I104" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J104" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K104" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L104" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M104" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=82591</t>
+        </is>
+      </c>
+      <c r="N104" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O104" s="11" t="inlineStr"/>
+      <c r="P104" s="11" t="inlineStr"/>
+    </row>
+    <row r="105" ht="40" customHeight="1">
+      <c r="A105" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR SULFATO, LAMIVUDINA</t>
+        </is>
+      </c>
+      <c r="C105" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA MACLEODS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 30 comprimidos (Blister Al/Al)</t>
+        </is>
+      </c>
+      <c r="D105" s="11" t="inlineStr">
+        <is>
+          <t>730479</t>
+        </is>
+      </c>
+      <c r="E105" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA MACLEODS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 30 comprimidos (Blister Al/Al)</t>
+        </is>
+      </c>
+      <c r="F105" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G105" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H105" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I105" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J105" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K105" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L105" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M105" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=85810</t>
+        </is>
+      </c>
+      <c r="N105" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O105" s="11" t="inlineStr"/>
+      <c r="P105" s="11" t="inlineStr"/>
+    </row>
+    <row r="106" ht="40" customHeight="1">
+      <c r="A106" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B106" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR SULFATO, LAMIVUDINA</t>
+        </is>
+      </c>
+      <c r="C106" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA TARBIS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG , 30 comprimidos (OPA/Al/PVC/Al)</t>
+        </is>
+      </c>
+      <c r="D106" s="11" t="inlineStr">
+        <is>
+          <t>733207</t>
+        </is>
+      </c>
+      <c r="E106" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA TARBIS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG , 30 comprimidos (OPA/Al/PVC/Al)</t>
+        </is>
+      </c>
+      <c r="F106" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G106" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H106" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I106" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J106" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K106" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L106" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M106" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=86488</t>
+        </is>
+      </c>
+      <c r="N106" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O106" s="11" t="inlineStr"/>
+      <c r="P106" s="11" t="inlineStr"/>
+    </row>
+    <row r="107" ht="40" customHeight="1">
+      <c r="A107" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR SULFATO, LAMIVUDINA</t>
+        </is>
+      </c>
+      <c r="C107" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA TARBIS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG , 30 comprimidos (PVC/PVDC/Al)</t>
+        </is>
+      </c>
+      <c r="D107" s="11" t="inlineStr">
+        <is>
+          <t>733208</t>
+        </is>
+      </c>
+      <c r="E107" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA TARBIS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG , 30 comprimidos (PVC/PVDC/Al)</t>
+        </is>
+      </c>
+      <c r="F107" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G107" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H107" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I107" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J107" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K107" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L107" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M107" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=86488</t>
+        </is>
+      </c>
+      <c r="N107" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O107" s="11" t="inlineStr"/>
+      <c r="P107" s="11" t="inlineStr"/>
+    </row>
+    <row r="108" ht="40" customHeight="1">
+      <c r="A108" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR, LAMIVUDINA</t>
+        </is>
+      </c>
+      <c r="C108" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA TEVA 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="D108" s="11" t="inlineStr">
+        <is>
+          <t>712262</t>
+        </is>
+      </c>
+      <c r="E108" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA TEVA 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="F108" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G108" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H108" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I108" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J108" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K108" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L108" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M108" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=81176</t>
+        </is>
+      </c>
+      <c r="N108" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O108" s="11" t="inlineStr"/>
+      <c r="P108" s="11" t="inlineStr"/>
+    </row>
+    <row r="109" ht="40" customHeight="1">
+      <c r="A109" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR SULFATO, LAMIVUDINA</t>
+        </is>
+      </c>
+      <c r="C109" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA VIATRIS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="D109" s="11" t="inlineStr">
+        <is>
+          <t>721596</t>
+        </is>
+      </c>
+      <c r="E109" s="11" t="inlineStr">
+        <is>
+          <t>ABACAVIR/LAMIVUDINA VIATRIS 600 MG/300 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="F109" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G109" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H109" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I109" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J109" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K109" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L109" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M109" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=83074</t>
+        </is>
+      </c>
+      <c r="N109" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O109" s="11" t="inlineStr"/>
+      <c r="P109" s="11" t="inlineStr"/>
+    </row>
+    <row r="110" ht="40" customHeight="1">
+      <c r="A110" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B110" s="11" t="inlineStr">
+        <is>
+          <t>INSULINA GLARGINA</t>
+        </is>
+      </c>
+      <c r="C110" s="11" t="inlineStr">
+        <is>
+          <t>ABASAGLAR 100 UNIDADES/ML KWIKPEN SOLUCION INYECTABLE EN PLUMA PRECARGADA  5 plumas precargadas de 3 ml</t>
+        </is>
+      </c>
+      <c r="D110" s="11" t="inlineStr">
+        <is>
+          <t>711261</t>
+        </is>
+      </c>
+      <c r="E110" s="11" t="inlineStr">
+        <is>
+          <t>ABASAGLAR 100 UNIDADES/ML KWIKPEN SOLUCION INYECTABLE EN PLUMA PRECARGADA  5 plumas precargadas de 3 ml</t>
+        </is>
+      </c>
+      <c r="F110" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G110" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H110" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I110" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J110" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K110" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L110" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M110" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=114944012</t>
+        </is>
+      </c>
+      <c r="N110" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O110" s="11" t="inlineStr"/>
+      <c r="P110" s="11" t="inlineStr"/>
+    </row>
+    <row r="111" ht="40" customHeight="1">
+      <c r="A111" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO</t>
+        </is>
+      </c>
+      <c r="C111" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 100 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 10 parches</t>
+        </is>
+      </c>
+      <c r="D111" s="11" t="inlineStr">
+        <is>
+          <t>765850</t>
+        </is>
+      </c>
+      <c r="E111" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 100 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 10 parches</t>
+        </is>
+      </c>
+      <c r="F111" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G111" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H111" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I111" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J111" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K111" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L111" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M111" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=74124</t>
+        </is>
+      </c>
+      <c r="N111" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O111" s="11" t="inlineStr"/>
+      <c r="P111" s="11" t="inlineStr"/>
+    </row>
+    <row r="112" ht="40" customHeight="1">
+      <c r="A112" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO</t>
+        </is>
+      </c>
+      <c r="C112" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 100 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 5 parches</t>
+        </is>
+      </c>
+      <c r="D112" s="11" t="inlineStr">
+        <is>
+          <t>680816</t>
+        </is>
+      </c>
+      <c r="E112" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 100 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 5 parches</t>
+        </is>
+      </c>
+      <c r="F112" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G112" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H112" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I112" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J112" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K112" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L112" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M112" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=74124</t>
+        </is>
+      </c>
+      <c r="N112" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O112" s="11" t="inlineStr"/>
+      <c r="P112" s="11" t="inlineStr"/>
+    </row>
+    <row r="113" ht="40" customHeight="1">
+      <c r="A113" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO</t>
+        </is>
+      </c>
+      <c r="C113" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 12 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 10 parches</t>
+        </is>
+      </c>
+      <c r="D113" s="11" t="inlineStr">
+        <is>
+          <t>765846</t>
+        </is>
+      </c>
+      <c r="E113" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 12 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 10 parches</t>
+        </is>
+      </c>
+      <c r="F113" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G113" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H113" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I113" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J113" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K113" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L113" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M113" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=74120</t>
+        </is>
+      </c>
+      <c r="N113" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O113" s="11" t="inlineStr"/>
+      <c r="P113" s="11" t="inlineStr"/>
+    </row>
+    <row r="114" ht="40" customHeight="1">
+      <c r="A114" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B114" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO</t>
+        </is>
+      </c>
+      <c r="C114" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 12 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 5 parches</t>
+        </is>
+      </c>
+      <c r="D114" s="11" t="inlineStr">
+        <is>
+          <t>680804</t>
+        </is>
+      </c>
+      <c r="E114" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 12 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 5 parches</t>
+        </is>
+      </c>
+      <c r="F114" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G114" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H114" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I114" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J114" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K114" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L114" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M114" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=74120</t>
+        </is>
+      </c>
+      <c r="N114" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O114" s="11" t="inlineStr"/>
+      <c r="P114" s="11" t="inlineStr"/>
+    </row>
+    <row r="115" ht="40" customHeight="1">
+      <c r="A115" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B115" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO</t>
+        </is>
+      </c>
+      <c r="C115" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 25 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 10 parches</t>
+        </is>
+      </c>
+      <c r="D115" s="11" t="inlineStr">
+        <is>
+          <t>765860</t>
+        </is>
+      </c>
+      <c r="E115" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 25 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 10 parches</t>
+        </is>
+      </c>
+      <c r="F115" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G115" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H115" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I115" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J115" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K115" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L115" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M115" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=74121</t>
+        </is>
+      </c>
+      <c r="N115" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O115" s="11" t="inlineStr"/>
+      <c r="P115" s="11" t="inlineStr"/>
+    </row>
+    <row r="116" ht="40" customHeight="1">
+      <c r="A116" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B116" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO</t>
+        </is>
+      </c>
+      <c r="C116" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 25 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 5 parches</t>
+        </is>
+      </c>
+      <c r="D116" s="11" t="inlineStr">
+        <is>
+          <t>680807</t>
+        </is>
+      </c>
+      <c r="E116" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 25 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 5 parches</t>
+        </is>
+      </c>
+      <c r="F116" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G116" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H116" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I116" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J116" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K116" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L116" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M116" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=74121</t>
+        </is>
+      </c>
+      <c r="N116" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O116" s="11" t="inlineStr"/>
+      <c r="P116" s="11" t="inlineStr"/>
+    </row>
+    <row r="117" ht="40" customHeight="1">
+      <c r="A117" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO</t>
+        </is>
+      </c>
+      <c r="C117" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 50 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 10 parches</t>
+        </is>
+      </c>
+      <c r="D117" s="11" t="inlineStr">
+        <is>
+          <t>765848</t>
+        </is>
+      </c>
+      <c r="E117" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 50 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 10 parches</t>
+        </is>
+      </c>
+      <c r="F117" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G117" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H117" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I117" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J117" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K117" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L117" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M117" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=74122</t>
+        </is>
+      </c>
+      <c r="N117" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O117" s="11" t="inlineStr"/>
+      <c r="P117" s="11" t="inlineStr"/>
+    </row>
+    <row r="118" ht="40" customHeight="1">
+      <c r="A118" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B118" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO</t>
+        </is>
+      </c>
+      <c r="C118" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 50 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 5 parches</t>
+        </is>
+      </c>
+      <c r="D118" s="11" t="inlineStr">
+        <is>
+          <t>680810</t>
+        </is>
+      </c>
+      <c r="E118" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 50 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 5 parches</t>
+        </is>
+      </c>
+      <c r="F118" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G118" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H118" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I118" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J118" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K118" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L118" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M118" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=74122</t>
+        </is>
+      </c>
+      <c r="N118" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O118" s="11" t="inlineStr"/>
+      <c r="P118" s="11" t="inlineStr"/>
+    </row>
+    <row r="119" ht="40" customHeight="1">
+      <c r="A119" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO</t>
+        </is>
+      </c>
+      <c r="C119" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 75 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 10 parches</t>
+        </is>
+      </c>
+      <c r="D119" s="11" t="inlineStr">
+        <is>
+          <t>765849</t>
+        </is>
+      </c>
+      <c r="E119" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 75 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 10 parches</t>
+        </is>
+      </c>
+      <c r="F119" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G119" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H119" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I119" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J119" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K119" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L119" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M119" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=74123</t>
+        </is>
+      </c>
+      <c r="N119" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O119" s="11" t="inlineStr"/>
+      <c r="P119" s="11" t="inlineStr"/>
+    </row>
+    <row r="120" ht="40" customHeight="1">
+      <c r="A120" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B120" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO</t>
+        </is>
+      </c>
+      <c r="C120" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 75 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 5 parches</t>
+        </is>
+      </c>
+      <c r="D120" s="11" t="inlineStr">
+        <is>
+          <t>680813</t>
+        </is>
+      </c>
+      <c r="E120" s="11" t="inlineStr">
+        <is>
+          <t>ABATTRA 75 MICROGRAMOS/HORA PARCHES TRANSDERMICOS EFG, 5 parches</t>
+        </is>
+      </c>
+      <c r="F120" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G120" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H120" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I120" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J120" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K120" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L120" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M120" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=74123</t>
+        </is>
+      </c>
+      <c r="N120" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O120" s="11" t="inlineStr"/>
+      <c r="P120" s="11" t="inlineStr"/>
+    </row>
+    <row r="121" ht="40" customHeight="1">
+      <c r="A121" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B121" s="11" t="inlineStr">
+        <is>
+          <t>SILDENAFILO CITRATO</t>
+        </is>
+      </c>
+      <c r="C121" s="11" t="inlineStr">
+        <is>
+          <t>ABECED 25 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 4 comprimidos</t>
+        </is>
+      </c>
+      <c r="D121" s="11" t="inlineStr">
+        <is>
+          <t>763340</t>
+        </is>
+      </c>
+      <c r="E121" s="11" t="inlineStr">
+        <is>
+          <t>ABECED 25 MG COMPRIMIDOS RECUBIERTOS CON PELICULA EFG, 4 comprimidos</t>
+        </is>
+      </c>
+      <c r="F121" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G121" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H121" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I121" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J121" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K121" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L121" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M121" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=89032</t>
+        </is>
+      </c>
+      <c r="N121" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O121" s="11" t="inlineStr"/>
+      <c r="P121" s="11" t="inlineStr"/>
+    </row>
+    <row r="122" ht="40" customHeight="1">
+      <c r="A122" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B122" s="11" t="inlineStr">
+        <is>
+          <t>LOPERAMIDA HIDROCLORURO</t>
+        </is>
+      </c>
+      <c r="C122" s="11" t="inlineStr">
+        <is>
+          <t>ABECLIN 2 MG COMPRIMIDOS EFG, 20 comprimidos</t>
+        </is>
+      </c>
+      <c r="D122" s="11" t="inlineStr">
+        <is>
+          <t>731848</t>
+        </is>
+      </c>
+      <c r="E122" s="11" t="inlineStr">
+        <is>
+          <t>ABECLIN 2 MG COMPRIMIDOS EFG, 20 comprimidos</t>
+        </is>
+      </c>
+      <c r="F122" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G122" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H122" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I122" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J122" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K122" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L122" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M122" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=86274</t>
+        </is>
+      </c>
+      <c r="N122" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O122" s="11" t="inlineStr"/>
+      <c r="P122" s="11" t="inlineStr"/>
+    </row>
+    <row r="123" ht="40" customHeight="1">
+      <c r="A123" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>IDECABTAGEN VICLEUCEL</t>
+        </is>
+      </c>
+      <c r="C123" s="11" t="inlineStr">
+        <is>
+          <t>ABECMA 260-500 x 10e6 CELULAS DISPERSION PARA PERFUSION, 1 o más bolsas</t>
+        </is>
+      </c>
+      <c r="D123" s="11" t="inlineStr">
+        <is>
+          <t>732577</t>
+        </is>
+      </c>
+      <c r="E123" s="11" t="inlineStr">
+        <is>
+          <t>ABECMA 260-500 x 10e6 CELULAS DISPERSION PARA PERFUSION, 1 o más bolsas</t>
+        </is>
+      </c>
+      <c r="F123" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G123" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H123" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I123" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J123" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K123" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L123" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M123" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=1211539001</t>
+        </is>
+      </c>
+      <c r="N123" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O123" s="11" t="inlineStr"/>
+      <c r="P123" s="11" t="inlineStr"/>
+    </row>
+    <row r="124" ht="40" customHeight="1">
+      <c r="A124" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
+        <is>
+          <t>AMFOTERICINA B</t>
+        </is>
+      </c>
+      <c r="C124" s="11" t="inlineStr">
+        <is>
+          <t>ABELCET COMPLEJO LIPIDICO 5 mg/ml CONCENTRADO PARA DISPERSION PARA PERFUSION , 10 viales de 20 ml</t>
+        </is>
+      </c>
+      <c r="D124" s="11" t="inlineStr">
+        <is>
+          <t>681726</t>
+        </is>
+      </c>
+      <c r="E124" s="11" t="inlineStr">
+        <is>
+          <t>ABELCET COMPLEJO LIPIDICO 5 mg/ml CONCENTRADO PARA DISPERSION PARA PERFUSION , 10 viales de 20 ml</t>
+        </is>
+      </c>
+      <c r="F124" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G124" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H124" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I124" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J124" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K124" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L124" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M124" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=60945</t>
+        </is>
+      </c>
+      <c r="N124" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O124" s="11" t="inlineStr"/>
+      <c r="P124" s="11" t="inlineStr"/>
+    </row>
+    <row r="125" ht="40" customHeight="1">
+      <c r="A125" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>BEVACIZUMAB</t>
+        </is>
+      </c>
+      <c r="C125" s="11" t="inlineStr">
+        <is>
+          <t>ABEVMY 25 MG/ML CONCENTRADO PARA SOLUCION PARA PERFUSION, 1 vial de 16 ml</t>
+        </is>
+      </c>
+      <c r="D125" s="11" t="inlineStr">
+        <is>
+          <t>764395</t>
+        </is>
+      </c>
+      <c r="E125" s="11" t="inlineStr">
+        <is>
+          <t>ABEVMY 25 MG/ML CONCENTRADO PARA SOLUCION PARA PERFUSION, 1 vial de 16 ml</t>
+        </is>
+      </c>
+      <c r="F125" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G125" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H125" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I125" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J125" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K125" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L125" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M125" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=1201515001</t>
+        </is>
+      </c>
+      <c r="N125" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O125" s="11" t="inlineStr"/>
+      <c r="P125" s="11" t="inlineStr"/>
+    </row>
+    <row r="126" ht="40" customHeight="1">
+      <c r="A126" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>BEVACIZUMAB</t>
+        </is>
+      </c>
+      <c r="C126" s="11" t="inlineStr">
+        <is>
+          <t>ABEVMY 25 MG/ML CONCENTRADO PARA SOLUCION PARA PERFUSION, 1 vial de 4 ml</t>
+        </is>
+      </c>
+      <c r="D126" s="11" t="inlineStr">
+        <is>
+          <t>764394</t>
+        </is>
+      </c>
+      <c r="E126" s="11" t="inlineStr">
+        <is>
+          <t>ABEVMY 25 MG/ML CONCENTRADO PARA SOLUCION PARA PERFUSION, 1 vial de 4 ml</t>
+        </is>
+      </c>
+      <c r="F126" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G126" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H126" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I126" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J126" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K126" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L126" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M126" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=1201515001</t>
+        </is>
+      </c>
+      <c r="N126" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O126" s="11" t="inlineStr"/>
+      <c r="P126" s="11" t="inlineStr"/>
+    </row>
+    <row r="127" ht="40" customHeight="1">
+      <c r="A127" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO CITRATO</t>
+        </is>
+      </c>
+      <c r="C127" s="11" t="inlineStr">
+        <is>
+          <t>ABFENTIQ 200 MICROGRAMOS COMPRIMIDOS PARA CHUPAR EFG 15 comprimidos</t>
+        </is>
+      </c>
+      <c r="D127" s="11" t="inlineStr">
+        <is>
+          <t>712741</t>
+        </is>
+      </c>
+      <c r="E127" s="11" t="inlineStr">
+        <is>
+          <t>ABFENTIQ 200 MICROGRAMOS COMPRIMIDOS PARA CHUPAR EFG 15 comprimidos</t>
+        </is>
+      </c>
+      <c r="F127" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G127" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H127" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I127" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J127" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K127" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L127" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M127" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=81256</t>
+        </is>
+      </c>
+      <c r="N127" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O127" s="11" t="inlineStr"/>
+      <c r="P127" s="11" t="inlineStr"/>
+    </row>
+    <row r="128" ht="40" customHeight="1">
+      <c r="A128" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B128" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO CITRATO</t>
+        </is>
+      </c>
+      <c r="C128" s="11" t="inlineStr">
+        <is>
+          <t>ABFENTIQ 200 MICROGRAMOS COMPRIMIDOS PARA CHUPAR EFG 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="D128" s="11" t="inlineStr">
+        <is>
+          <t>712742</t>
+        </is>
+      </c>
+      <c r="E128" s="11" t="inlineStr">
+        <is>
+          <t>ABFENTIQ 200 MICROGRAMOS COMPRIMIDOS PARA CHUPAR EFG 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="F128" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G128" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H128" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I128" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J128" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K128" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L128" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M128" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=81256</t>
+        </is>
+      </c>
+      <c r="N128" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O128" s="11" t="inlineStr"/>
+      <c r="P128" s="11" t="inlineStr"/>
+    </row>
+    <row r="129" ht="40" customHeight="1">
+      <c r="A129" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO CITRATO</t>
+        </is>
+      </c>
+      <c r="C129" s="11" t="inlineStr">
+        <is>
+          <t>ABFENTIQ 400 MICROGRAMOS COMPRIMIDOS PARA CHUPAR EFG 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="D129" s="11" t="inlineStr">
+        <is>
+          <t>712746</t>
+        </is>
+      </c>
+      <c r="E129" s="11" t="inlineStr">
+        <is>
+          <t>ABFENTIQ 400 MICROGRAMOS COMPRIMIDOS PARA CHUPAR EFG 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="F129" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G129" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H129" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I129" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J129" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K129" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L129" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M129" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=81257</t>
+        </is>
+      </c>
+      <c r="N129" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O129" s="11" t="inlineStr"/>
+      <c r="P129" s="11" t="inlineStr"/>
+    </row>
+    <row r="130" ht="40" customHeight="1">
+      <c r="A130" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B130" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO CITRATO</t>
+        </is>
+      </c>
+      <c r="C130" s="11" t="inlineStr">
+        <is>
+          <t>ABFENTIQ 600 MICROGRAMOS COMPRIMIDOS PARA CHUPAR EFG 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="D130" s="11" t="inlineStr">
+        <is>
+          <t>712749</t>
+        </is>
+      </c>
+      <c r="E130" s="11" t="inlineStr">
+        <is>
+          <t>ABFENTIQ 600 MICROGRAMOS COMPRIMIDOS PARA CHUPAR EFG 30 comprimidos</t>
+        </is>
+      </c>
+      <c r="F130" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G130" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H130" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I130" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J130" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K130" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L130" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M130" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=81258</t>
+        </is>
+      </c>
+      <c r="N130" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O130" s="11" t="inlineStr"/>
+      <c r="P130" s="11" t="inlineStr"/>
+    </row>
+    <row r="131" ht="40" customHeight="1">
+      <c r="A131" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B131" s="11" t="inlineStr">
+        <is>
+          <t>FENTANILO CITRATO</t>
+        </is>
+      </c>
+      <c r="C131" s="11" t="inlineStr">
+        <is>
+          <t>ABFENTIQ 800 MICROGRAMOS COMPRIMIDOS PARA CHUPAR EFG 15 comprimidos</t>
+        </is>
+      </c>
+      <c r="D131" s="11" t="inlineStr">
+        <is>
+          <t>712751</t>
+        </is>
+      </c>
+      <c r="E131" s="11" t="inlineStr">
+        <is>
+          <t>ABFENTIQ 800 MICROGRAMOS COMPRIMIDOS PARA CHUPAR EFG 15 comprimidos</t>
+        </is>
+      </c>
+      <c r="F131" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G131" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H131" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I131" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J131" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K131" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L131" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M131" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=81259</t>
+        </is>
+      </c>
+      <c r="N131" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O131" s="11" t="inlineStr"/>
+      <c r="P131" s="11" t="inlineStr"/>
+    </row>
+    <row r="132" ht="40" customHeight="1">
+      <c r="A132" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B132" s="11" t="inlineStr">
+        <is>
+          <t>FLUOCINOLONA ACETONIDO, FRAMICETINA SULFATO</t>
+        </is>
+      </c>
+      <c r="C132" s="11" t="inlineStr">
+        <is>
+          <t>ABICREM 0,25 MG/G +5 MG/G CREMA , 1 tubo de 50 g</t>
+        </is>
+      </c>
+      <c r="D132" s="11" t="inlineStr">
+        <is>
+          <t>700286</t>
+        </is>
+      </c>
+      <c r="E132" s="11" t="inlineStr">
+        <is>
+          <t>ABICREM 0,25 MG/G +5 MG/G CREMA , 1 tubo de 50 g</t>
+        </is>
+      </c>
+      <c r="F132" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G132" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H132" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I132" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J132" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K132" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L132" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M132" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=49840</t>
+        </is>
+      </c>
+      <c r="N132" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O132" s="11" t="inlineStr"/>
+      <c r="P132" s="11" t="inlineStr"/>
+    </row>
+    <row r="133" ht="40" customHeight="1">
+      <c r="A133" s="12" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B133" s="12" t="inlineStr"/>
+      <c r="C133" s="12" t="inlineStr">
+        <is>
+          <t>ABIES NIGRA GLOBULOS BOIRON, 1 envase de 4g (C5)</t>
+        </is>
+      </c>
+      <c r="D133" s="12" t="inlineStr">
+        <is>
+          <t>734308</t>
+        </is>
+      </c>
+      <c r="E133" s="12" t="inlineStr">
+        <is>
+          <t>ABIES NIGRA GLOBULOS BOIRON, 1 envase de 4g (C5)</t>
+        </is>
+      </c>
+      <c r="F133" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 100-200 µg si cal
+D.màx: 200 µg/6h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G133" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H133" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I133" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J133" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K133" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L133" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M133" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=86829</t>
+        </is>
+      </c>
+      <c r="N133" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O133" s="12" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="P133" s="12" t="inlineStr"/>
+    </row>
+    <row r="134" ht="40" customHeight="1">
+      <c r="A134" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B134" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C134" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 1 MG/ML SOLUCION ORAL EFG , 150 ml</t>
+        </is>
+      </c>
+      <c r="D134" s="11" t="inlineStr">
+        <is>
+          <t>709769</t>
+        </is>
+      </c>
+      <c r="E134" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 1 MG/ML SOLUCION ORAL EFG , 150 ml</t>
+        </is>
+      </c>
+      <c r="F134" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G134" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H134" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I134" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J134" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K134" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L134" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M134" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=80580</t>
+        </is>
+      </c>
+      <c r="N134" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O134" s="11" t="inlineStr"/>
+      <c r="P134" s="11" t="inlineStr"/>
+    </row>
+    <row r="135" ht="40" customHeight="1">
+      <c r="A135" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B135" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C135" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 10 MG COMPRIMIDOS BUCODISPERSABLES EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="D135" s="11" t="inlineStr">
+        <is>
+          <t>704003</t>
+        </is>
+      </c>
+      <c r="E135" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 10 MG COMPRIMIDOS BUCODISPERSABLES EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="F135" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G135" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H135" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I135" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J135" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K135" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L135" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M135" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=79154</t>
+        </is>
+      </c>
+      <c r="N135" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O135" s="11" t="inlineStr"/>
+      <c r="P135" s="11" t="inlineStr"/>
+    </row>
+    <row r="136" ht="40" customHeight="1">
+      <c r="A136" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B136" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C136" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 10 MG COMPRIMIDOS EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="D136" s="11" t="inlineStr">
+        <is>
+          <t>704000</t>
+        </is>
+      </c>
+      <c r="E136" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 10 MG COMPRIMIDOS EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="F136" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G136" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H136" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I136" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J136" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K136" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L136" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M136" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=79151</t>
+        </is>
+      </c>
+      <c r="N136" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O136" s="11" t="inlineStr"/>
+      <c r="P136" s="11" t="inlineStr"/>
+    </row>
+    <row r="137" ht="40" customHeight="1">
+      <c r="A137" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B137" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C137" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 15 MG COMPRIMIDOS BUCODISPERSABLES EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="D137" s="11" t="inlineStr">
+        <is>
+          <t>704004</t>
+        </is>
+      </c>
+      <c r="E137" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 15 MG COMPRIMIDOS BUCODISPERSABLES EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="F137" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G137" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H137" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I137" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J137" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K137" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L137" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M137" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=79155</t>
+        </is>
+      </c>
+      <c r="N137" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O137" s="11" t="inlineStr"/>
+      <c r="P137" s="11" t="inlineStr"/>
+    </row>
+    <row r="138" ht="40" customHeight="1">
+      <c r="A138" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B138" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C138" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 15 MG COMPRIMIDOS EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="D138" s="11" t="inlineStr">
+        <is>
+          <t>704001</t>
+        </is>
+      </c>
+      <c r="E138" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 15 MG COMPRIMIDOS EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="F138" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G138" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H138" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I138" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J138" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K138" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L138" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M138" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=79152</t>
+        </is>
+      </c>
+      <c r="N138" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O138" s="11" t="inlineStr"/>
+      <c r="P138" s="11" t="inlineStr"/>
+    </row>
+    <row r="139" ht="40" customHeight="1">
+      <c r="A139" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B139" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C139" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 30 MG COMPRIMIDOS EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="D139" s="11" t="inlineStr">
+        <is>
+          <t>704002</t>
+        </is>
+      </c>
+      <c r="E139" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 30 MG COMPRIMIDOS EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="F139" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G139" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H139" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I139" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J139" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K139" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L139" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M139" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=79153</t>
+        </is>
+      </c>
+      <c r="N139" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O139" s="11" t="inlineStr"/>
+      <c r="P139" s="11" t="inlineStr"/>
+    </row>
+    <row r="140" ht="40" customHeight="1">
+      <c r="A140" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B140" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C140" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 5 MG COMPRIMIDOS EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="D140" s="11" t="inlineStr">
+        <is>
+          <t>703999</t>
+        </is>
+      </c>
+      <c r="E140" s="11" t="inlineStr">
+        <is>
+          <t>ABIK 5 MG COMPRIMIDOS EFG , 28 comprimidos</t>
+        </is>
+      </c>
+      <c r="F140" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G140" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H140" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I140" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J140" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K140" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L140" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M140" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=79150</t>
+        </is>
+      </c>
+      <c r="N140" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O140" s="11" t="inlineStr"/>
+      <c r="P140" s="11" t="inlineStr"/>
+    </row>
+    <row r="141" ht="40" customHeight="1">
+      <c r="A141" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B141" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C141" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 300 MG POLVO Y DISOLVENTE PARA SUSPENSION INYECTABLE DE LIBERACION PROLONGADA, 1 vial + 1 vial de disolvente</t>
+        </is>
+      </c>
+      <c r="D141" s="11" t="inlineStr">
+        <is>
+          <t>701735</t>
+        </is>
+      </c>
+      <c r="E141" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 300 MG POLVO Y DISOLVENTE PARA SUSPENSION INYECTABLE DE LIBERACION PROLONGADA, 1 vial + 1 vial de disolvente</t>
+        </is>
+      </c>
+      <c r="F141" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G141" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H141" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I141" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J141" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K141" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L141" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M141" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=113882001</t>
+        </is>
+      </c>
+      <c r="N141" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O141" s="11" t="inlineStr"/>
+      <c r="P141" s="11" t="inlineStr"/>
+    </row>
+    <row r="142" ht="40" customHeight="1">
+      <c r="A142" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B142" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C142" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 400 MG POLVO Y DISOLVENTE PARA SUSPENSION INYECTABLE DE LIBERACION PROLONGADA, 1 vial + 1 vial de disolvente</t>
+        </is>
+      </c>
+      <c r="D142" s="11" t="inlineStr">
+        <is>
+          <t>701736</t>
+        </is>
+      </c>
+      <c r="E142" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 400 MG POLVO Y DISOLVENTE PARA SUSPENSION INYECTABLE DE LIBERACION PROLONGADA, 1 vial + 1 vial de disolvente</t>
+        </is>
+      </c>
+      <c r="F142" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G142" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H142" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I142" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J142" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K142" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L142" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M142" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=113882002</t>
+        </is>
+      </c>
+      <c r="N142" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O142" s="11" t="inlineStr"/>
+      <c r="P142" s="11" t="inlineStr"/>
+    </row>
+    <row r="143" ht="40" customHeight="1">
+      <c r="A143" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B143" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C143" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 400 MG POLVO Y DISOLVENTE PARA SUSPENSION INYECTABLE DE LIBERACION PROLONGADA, 1 vial + 1 vial de disolvente</t>
+        </is>
+      </c>
+      <c r="D143" s="11" t="inlineStr">
+        <is>
+          <t>763460</t>
+        </is>
+      </c>
+      <c r="E143" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 400 MG POLVO Y DISOLVENTE PARA SUSPENSION INYECTABLE DE LIBERACION PROLONGADA, 1 vial + 1 vial de disolvente</t>
+        </is>
+      </c>
+      <c r="F143" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G143" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H143" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I143" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J143" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K143" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L143" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M143" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=113882002IP</t>
+        </is>
+      </c>
+      <c r="N143" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O143" s="11" t="inlineStr"/>
+      <c r="P143" s="11" t="inlineStr"/>
+    </row>
+    <row r="144" ht="40" customHeight="1">
+      <c r="A144" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B144" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C144" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 400 MG POLVO Y DISOLVENTE PARA SUSPENSION INYECTABLE DE LIBERACION PROLONGADA, 1 vial + 1 vial de disolvente</t>
+        </is>
+      </c>
+      <c r="D144" s="11" t="inlineStr">
+        <is>
+          <t>763693</t>
+        </is>
+      </c>
+      <c r="E144" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 400 MG POLVO Y DISOLVENTE PARA SUSPENSION INYECTABLE DE LIBERACION PROLONGADA, 1 vial + 1 vial de disolvente</t>
+        </is>
+      </c>
+      <c r="F144" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G144" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H144" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I144" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J144" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K144" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L144" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M144" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=113882002IP1</t>
+        </is>
+      </c>
+      <c r="N144" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O144" s="11" t="inlineStr"/>
+      <c r="P144" s="11" t="inlineStr"/>
+    </row>
+    <row r="145" ht="40" customHeight="1">
+      <c r="A145" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B145" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL</t>
+        </is>
+      </c>
+      <c r="C145" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 400 MG POLVO Y DISOLVENTE PARA SUSPENSION INYECTABLE DE LIBERACION PROLONGADA, 1 vial + 1 vial de disolvente</t>
+        </is>
+      </c>
+      <c r="D145" s="11" t="inlineStr">
+        <is>
+          <t>768547</t>
+        </is>
+      </c>
+      <c r="E145" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 400 MG POLVO Y DISOLVENTE PARA SUSPENSION INYECTABLE DE LIBERACION PROLONGADA, 1 vial + 1 vial de disolvente</t>
+        </is>
+      </c>
+      <c r="F145" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G145" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H145" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I145" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J145" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K145" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L145" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M145" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=113882002IP2</t>
+        </is>
+      </c>
+      <c r="N145" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O145" s="11" t="inlineStr"/>
+      <c r="P145" s="11" t="inlineStr"/>
+    </row>
+    <row r="146" ht="40" customHeight="1">
+      <c r="A146" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B146" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL MONOHIDRATO</t>
+        </is>
+      </c>
+      <c r="C146" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 720 MG SUSPENSION INYECTABLE DE LIBERACIÓN PROLONGADA EN JERINGA PRECARGADA, 1 jeringa de 2,4 ml</t>
+        </is>
+      </c>
+      <c r="D146" s="11" t="inlineStr">
+        <is>
+          <t>764868</t>
+        </is>
+      </c>
+      <c r="E146" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 720 MG SUSPENSION INYECTABLE DE LIBERACIÓN PROLONGADA EN JERINGA PRECARGADA, 1 jeringa de 2,4 ml</t>
+        </is>
+      </c>
+      <c r="F146" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G146" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H146" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I146" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J146" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K146" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L146" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M146" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=113882009</t>
+        </is>
+      </c>
+      <c r="N146" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O146" s="11" t="inlineStr"/>
+      <c r="P146" s="11" t="inlineStr"/>
+    </row>
+    <row r="147" ht="40" customHeight="1">
+      <c r="A147" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B147" s="11" t="inlineStr">
+        <is>
+          <t>ARIPIPRAZOL MONOHIDRATO</t>
+        </is>
+      </c>
+      <c r="C147" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 960 MG SUSPENSION INYECTABLE DE LIBERACION PROLONGADA EN JERINGA PRECARGADA, 1 jeringa de 3,2 ml</t>
+        </is>
+      </c>
+      <c r="D147" s="11" t="inlineStr">
+        <is>
+          <t>764869</t>
+        </is>
+      </c>
+      <c r="E147" s="11" t="inlineStr">
+        <is>
+          <t>ABILIFY MAINTENA 960 MG SUSPENSION INYECTABLE DE LIBERACION PROLONGADA EN JERINGA PRECARGADA, 1 jeringa de 3,2 ml</t>
+        </is>
+      </c>
+      <c r="F147" s="11" t="inlineStr">
+        <is>
+          <t>PENDENT — consultar fitxa CIMA</t>
+        </is>
+      </c>
+      <c r="G147" s="11" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H147" s="11" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I147" s="11" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J147" s="11" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K147" s="11" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L147" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="M147" s="11" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=113882010</t>
+        </is>
+      </c>
+      <c r="N147" s="11" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O147" s="11" t="inlineStr"/>
+      <c r="P147" s="11" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:P97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7048,17 +10768,13 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>COLUMNES AUTOMÀTIQUES (omplertes pel script)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7228,17 +10944,13 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
           <t>COLUMNES DE VALIDACIÓ CLÍNICA (les omples tu)</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -7264,17 +10976,13 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
-    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
           <t>COLORS DE FILES</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7324,17 +11032,13 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr"/>
-    </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
           <t>QUAN EL SCRIPT DETECTA UN FÀRMAC NOU</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">

</xml_diff>

<commit_message>
Novetats CIMA: 28 nous farmacos pendents de validacio
</commit_message>
<xml_diff>
--- a/inhaladors_MPOC_ASMA_Avanzado_FINAL.xlsx
+++ b/inhaladors_MPOC_ASMA_Avanzado_FINAL.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P347"/>
+  <dimension ref="A1:P375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -26424,6 +26424,2202 @@
       <c r="O347" s="12" t="inlineStr"/>
       <c r="P347" s="12" t="inlineStr"/>
     </row>
+    <row r="348" ht="40" customHeight="1">
+      <c r="A348" s="12" t="inlineStr">
+        <is>
+          <t>LABA/GCI</t>
+        </is>
+      </c>
+      <c r="B348" s="12" t="inlineStr">
+        <is>
+          <t>fluticasona</t>
+        </is>
+      </c>
+      <c r="C348" s="12" t="inlineStr">
+        <is>
+          <t>REVINTY ELLIPTA 92 MICROGRAMOS/22 MICROGRAMOS POLVO PARA INHALACION (UNIDOSIS), 1 inhalador de 30 dosis</t>
+        </is>
+      </c>
+      <c r="D348" s="12" t="inlineStr">
+        <is>
+          <t>768316</t>
+        </is>
+      </c>
+      <c r="E348" s="12" t="inlineStr">
+        <is>
+          <t>REVINTY ELLIPTA 92 MICROGRAMOS/22 MICROGRAMOS POLVO PARA INHALACION (UNIDOSIS), 1 inhalador de 30 dosis</t>
+        </is>
+      </c>
+      <c r="F348" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 250-500 µg/12h
+D.màx: 500 µg/12h
+Asma baixa: 100-250 µg/24h
+Asma mitjana: 251-500 µg/24h
+Asma alta: 501-1.000 µg/24h</t>
+        </is>
+      </c>
+      <c r="G348" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H348" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I348" s="12" t="inlineStr">
+        <is>
+          <t>&lt;50 l/m</t>
+        </is>
+      </c>
+      <c r="J348" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K348" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11818</t>
+        </is>
+      </c>
+      <c r="L348" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M348" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=114929002IP</t>
+        </is>
+      </c>
+      <c r="N348" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O348" s="12" t="inlineStr"/>
+      <c r="P348" s="12" t="inlineStr"/>
+    </row>
+    <row r="349" ht="40" customHeight="1">
+      <c r="A349" s="12" t="inlineStr">
+        <is>
+          <t>LABA/GCI</t>
+        </is>
+      </c>
+      <c r="B349" s="12" t="inlineStr">
+        <is>
+          <t>fluticasona</t>
+        </is>
+      </c>
+      <c r="C349" s="12" t="inlineStr">
+        <is>
+          <t>REVINTY ELLIPTA 92 MICROGRAMOS/22 MICROGRAMOS POLVO PARA INHALACION (UNIDOSIS), 1 inhalador de 30 dosis</t>
+        </is>
+      </c>
+      <c r="D349" s="12" t="inlineStr">
+        <is>
+          <t>769953</t>
+        </is>
+      </c>
+      <c r="E349" s="12" t="inlineStr">
+        <is>
+          <t>REVINTY ELLIPTA 92 MICROGRAMOS/22 MICROGRAMOS POLVO PARA INHALACION (UNIDOSIS), 1 inhalador de 30 dosis</t>
+        </is>
+      </c>
+      <c r="F349" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 250-500 µg/12h
+D.màx: 500 µg/12h
+Asma baixa: 100-250 µg/24h
+Asma mitjana: 251-500 µg/24h
+Asma alta: 501-1.000 µg/24h</t>
+        </is>
+      </c>
+      <c r="G349" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H349" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I349" s="12" t="inlineStr">
+        <is>
+          <t>&lt;50 l/m</t>
+        </is>
+      </c>
+      <c r="J349" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K349" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11818</t>
+        </is>
+      </c>
+      <c r="L349" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M349" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=114929002IP1</t>
+        </is>
+      </c>
+      <c r="N349" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O349" s="12" t="inlineStr"/>
+      <c r="P349" s="12" t="inlineStr"/>
+    </row>
+    <row r="350" ht="40" customHeight="1">
+      <c r="A350" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B350" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C350" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA ALDO-UNION 0,25 mg/ml SUSPENSION PARA INHALACION POR NEBULIZADOR , 20 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="D350" s="12" t="inlineStr">
+        <is>
+          <t>651628</t>
+        </is>
+      </c>
+      <c r="E350" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA ALDO-UNION 0,25 mg/ml SUSPENSION PARA INHALACION POR NEBULIZADOR , 20 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="F350" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G350" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H350" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I350" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J350" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K350" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L350" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M350" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=66943</t>
+        </is>
+      </c>
+      <c r="N350" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O350" s="12" t="inlineStr"/>
+      <c r="P350" s="12" t="inlineStr"/>
+    </row>
+    <row r="351" ht="40" customHeight="1">
+      <c r="A351" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B351" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C351" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA ALDO-UNION 0,5 mg/ml SUSPENSION PARA INHALACION POR NEBULIZADOR , 20 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="D351" s="12" t="inlineStr">
+        <is>
+          <t>651626</t>
+        </is>
+      </c>
+      <c r="E351" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA ALDO-UNION 0,5 mg/ml SUSPENSION PARA INHALACION POR NEBULIZADOR , 20 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="F351" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G351" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H351" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I351" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J351" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K351" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L351" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M351" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=66942</t>
+        </is>
+      </c>
+      <c r="N351" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O351" s="12" t="inlineStr"/>
+      <c r="P351" s="12" t="inlineStr"/>
+    </row>
+    <row r="352" ht="40" customHeight="1">
+      <c r="A352" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B352" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C352" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA ALDO-UNION 100 MICROGRAMOS/PULSACION SUSPENSION PARA INHALACION EN ENVASE A PRESION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D352" s="12" t="inlineStr">
+        <is>
+          <t>725241</t>
+        </is>
+      </c>
+      <c r="E352" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA ALDO-UNION 100 MICROGRAMOS/PULSACION SUSPENSION PARA INHALACION EN ENVASE A PRESION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F352" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G352" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H352" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I352" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J352" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K352" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L352" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M352" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=83987</t>
+        </is>
+      </c>
+      <c r="N352" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O352" s="12" t="inlineStr"/>
+      <c r="P352" s="12" t="inlineStr"/>
+    </row>
+    <row r="353" ht="40" customHeight="1">
+      <c r="A353" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B353" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C353" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA ALDO-UNION 200 microgramos/pulsación SUSPENSIÓN PARA INHALACIÓN EN ENVASE A PRESIÓN, 1 inhalador de 120 dosis</t>
+        </is>
+      </c>
+      <c r="D353" s="12" t="inlineStr">
+        <is>
+          <t>672718</t>
+        </is>
+      </c>
+      <c r="E353" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA ALDO-UNION 200 microgramos/pulsación SUSPENSIÓN PARA INHALACIÓN EN ENVASE A PRESIÓN, 1 inhalador de 120 dosis</t>
+        </is>
+      </c>
+      <c r="F353" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G353" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H353" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I353" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J353" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K353" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L353" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M353" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=61664</t>
+        </is>
+      </c>
+      <c r="N353" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O353" s="12" t="inlineStr"/>
+      <c r="P353" s="12" t="inlineStr"/>
+    </row>
+    <row r="354" ht="40" customHeight="1">
+      <c r="A354" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B354" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C354" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA ALDO-UNION 200 microgramos/pulsación SUSPENSIÓN PARA INHALACIÓN EN ENVASE A PRESIÓN, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D354" s="12" t="inlineStr">
+        <is>
+          <t>799015</t>
+        </is>
+      </c>
+      <c r="E354" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA ALDO-UNION 200 microgramos/pulsación SUSPENSIÓN PARA INHALACIÓN EN ENVASE A PRESIÓN, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F354" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G354" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H354" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I354" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J354" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K354" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L354" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M354" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=61664</t>
+        </is>
+      </c>
+      <c r="N354" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O354" s="12" t="inlineStr"/>
+      <c r="P354" s="12" t="inlineStr"/>
+    </row>
+    <row r="355" ht="40" customHeight="1">
+      <c r="A355" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B355" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C355" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA  ALDO-UNION 50 microgramos/pulsación SUSPENSIÓN PARA INHALACIÓN EN ENVASE A PRESIÓN , 1 envase aerosol de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D355" s="12" t="inlineStr">
+        <is>
+          <t>668905</t>
+        </is>
+      </c>
+      <c r="E355" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA  ALDO-UNION 50 microgramos/pulsación SUSPENSIÓN PARA INHALACIÓN EN ENVASE A PRESIÓN , 1 envase aerosol de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F355" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G355" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H355" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I355" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J355" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K355" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L355" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M355" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=61663</t>
+        </is>
+      </c>
+      <c r="N355" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O355" s="12" t="inlineStr"/>
+      <c r="P355" s="12" t="inlineStr"/>
+    </row>
+    <row r="356" ht="40" customHeight="1">
+      <c r="A356" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B356" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C356" s="12" t="inlineStr">
+        <is>
+          <t>PULMICORT TURBUHALER 100 microgramos/inhalacion POLVO PARA INHALACION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D356" s="12" t="inlineStr">
+        <is>
+          <t>660910</t>
+        </is>
+      </c>
+      <c r="E356" s="12" t="inlineStr">
+        <is>
+          <t>PULMICORT TURBUHALER 100 microgramos/inhalacion POLVO PARA INHALACION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F356" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G356" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H356" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I356" s="12" t="inlineStr">
+        <is>
+          <t>50-60 l/m</t>
+        </is>
+      </c>
+      <c r="J356" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K356" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11893</t>
+        </is>
+      </c>
+      <c r="L356" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M356" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=62046</t>
+        </is>
+      </c>
+      <c r="N356" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O356" s="12" t="inlineStr"/>
+      <c r="P356" s="12" t="inlineStr"/>
+    </row>
+    <row r="357" ht="40" customHeight="1">
+      <c r="A357" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B357" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C357" s="12" t="inlineStr">
+        <is>
+          <t>PULMICORT TURBUHALER 200 microgramos/inhalación POLVO PARA INHALACION, 1 inhalador de 100 dosis</t>
+        </is>
+      </c>
+      <c r="D357" s="12" t="inlineStr">
+        <is>
+          <t>651927</t>
+        </is>
+      </c>
+      <c r="E357" s="12" t="inlineStr">
+        <is>
+          <t>PULMICORT TURBUHALER 200 microgramos/inhalación POLVO PARA INHALACION, 1 inhalador de 100 dosis</t>
+        </is>
+      </c>
+      <c r="F357" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G357" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H357" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I357" s="12" t="inlineStr">
+        <is>
+          <t>50-60 l/m</t>
+        </is>
+      </c>
+      <c r="J357" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K357" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11893</t>
+        </is>
+      </c>
+      <c r="L357" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M357" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=59254</t>
+        </is>
+      </c>
+      <c r="N357" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O357" s="12" t="inlineStr"/>
+      <c r="P357" s="12" t="inlineStr"/>
+    </row>
+    <row r="358" ht="40" customHeight="1">
+      <c r="A358" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B358" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C358" s="12" t="inlineStr">
+        <is>
+          <t>PULMICORT TURBUHALER 400 microgramos/inhalación POLVO PARA INHALACION, 1 inhalador de 100 dosis</t>
+        </is>
+      </c>
+      <c r="D358" s="12" t="inlineStr">
+        <is>
+          <t>885640</t>
+        </is>
+      </c>
+      <c r="E358" s="12" t="inlineStr">
+        <is>
+          <t>PULMICORT TURBUHALER 400 microgramos/inhalación POLVO PARA INHALACION, 1 inhalador de 100 dosis</t>
+        </is>
+      </c>
+      <c r="F358" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G358" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H358" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I358" s="12" t="inlineStr">
+        <is>
+          <t>50-60 l/m</t>
+        </is>
+      </c>
+      <c r="J358" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K358" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11893</t>
+        </is>
+      </c>
+      <c r="L358" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M358" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=59255</t>
+        </is>
+      </c>
+      <c r="N358" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O358" s="12" t="inlineStr"/>
+      <c r="P358" s="12" t="inlineStr"/>
+    </row>
+    <row r="359" ht="40" customHeight="1">
+      <c r="A359" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B359" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C359" s="12" t="inlineStr">
+        <is>
+          <t>PULMICORT 0,25 mg/ml SUSPENSION PARA INHALACION POR  NEBULIZADOR, 5 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="D359" s="12" t="inlineStr">
+        <is>
+          <t>901199</t>
+        </is>
+      </c>
+      <c r="E359" s="12" t="inlineStr">
+        <is>
+          <t>PULMICORT 0,25 mg/ml SUSPENSION PARA INHALACION POR  NEBULIZADOR, 5 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="F359" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G359" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H359" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I359" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J359" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K359" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L359" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M359" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=59298</t>
+        </is>
+      </c>
+      <c r="N359" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O359" s="12" t="inlineStr"/>
+      <c r="P359" s="12" t="inlineStr"/>
+    </row>
+    <row r="360" ht="40" customHeight="1">
+      <c r="A360" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B360" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C360" s="12" t="inlineStr">
+        <is>
+          <t>PULMICORT 0,50 mg/ml SUSPENSION PARA INHALACION POR NEBULIZADOR, 5 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="D360" s="12" t="inlineStr">
+        <is>
+          <t>901082</t>
+        </is>
+      </c>
+      <c r="E360" s="12" t="inlineStr">
+        <is>
+          <t>PULMICORT 0,50 mg/ml SUSPENSION PARA INHALACION POR NEBULIZADOR, 5 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="F360" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G360" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H360" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I360" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J360" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K360" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L360" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M360" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=59297</t>
+        </is>
+      </c>
+      <c r="N360" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O360" s="12" t="inlineStr"/>
+      <c r="P360" s="12" t="inlineStr"/>
+    </row>
+    <row r="361" ht="40" customHeight="1">
+      <c r="A361" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B361" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C361" s="12" t="inlineStr">
+        <is>
+          <t>BUDENA 0,25 MG/ML SUSPENSION PARA INHALACION POR NEBULIZADOR, 20 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="D361" s="12" t="inlineStr">
+        <is>
+          <t>728863</t>
+        </is>
+      </c>
+      <c r="E361" s="12" t="inlineStr">
+        <is>
+          <t>BUDENA 0,25 MG/ML SUSPENSION PARA INHALACION POR NEBULIZADOR, 20 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="F361" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G361" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H361" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I361" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J361" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K361" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L361" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M361" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=85219</t>
+        </is>
+      </c>
+      <c r="N361" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O361" s="12" t="inlineStr"/>
+      <c r="P361" s="12" t="inlineStr"/>
+    </row>
+    <row r="362" ht="40" customHeight="1">
+      <c r="A362" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B362" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C362" s="12" t="inlineStr">
+        <is>
+          <t>BUDENA 0,5 MG/ML SUSPENSION PARA INHALACION POR NEBULIZADOR, 20 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="D362" s="12" t="inlineStr">
+        <is>
+          <t>728864</t>
+        </is>
+      </c>
+      <c r="E362" s="12" t="inlineStr">
+        <is>
+          <t>BUDENA 0,5 MG/ML SUSPENSION PARA INHALACION POR NEBULIZADOR, 20 ampollas de 2 ml</t>
+        </is>
+      </c>
+      <c r="F362" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G362" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H362" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I362" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J362" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K362" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L362" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M362" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=85220</t>
+        </is>
+      </c>
+      <c r="N362" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O362" s="12" t="inlineStr"/>
+      <c r="P362" s="12" t="inlineStr"/>
+    </row>
+    <row r="363" ht="40" customHeight="1">
+      <c r="A363" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B363" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C363" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA EASYHALER 100 microgramos POLVO PARA INHALACION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D363" s="12" t="inlineStr">
+        <is>
+          <t>650966</t>
+        </is>
+      </c>
+      <c r="E363" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA EASYHALER 100 microgramos POLVO PARA INHALACION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F363" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G363" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H363" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I363" s="12" t="inlineStr">
+        <is>
+          <t>&lt;50 l/m</t>
+        </is>
+      </c>
+      <c r="J363" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K363" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11817</t>
+        </is>
+      </c>
+      <c r="L363" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M363" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=66670</t>
+        </is>
+      </c>
+      <c r="N363" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O363" s="12" t="inlineStr"/>
+      <c r="P363" s="12" t="inlineStr"/>
+    </row>
+    <row r="364" ht="40" customHeight="1">
+      <c r="A364" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B364" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C364" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA EASYHALER 200 mcg POLVO PARA INHALACION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D364" s="12" t="inlineStr">
+        <is>
+          <t>650965</t>
+        </is>
+      </c>
+      <c r="E364" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA EASYHALER 200 mcg POLVO PARA INHALACION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F364" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G364" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H364" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I364" s="12" t="inlineStr">
+        <is>
+          <t>&lt;50 l/m</t>
+        </is>
+      </c>
+      <c r="J364" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K364" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11817</t>
+        </is>
+      </c>
+      <c r="L364" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M364" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=66669</t>
+        </is>
+      </c>
+      <c r="N364" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O364" s="12" t="inlineStr"/>
+      <c r="P364" s="12" t="inlineStr"/>
+    </row>
+    <row r="365" ht="40" customHeight="1">
+      <c r="A365" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B365" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C365" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA EASYHALER 400 microgramos POLVO PARA INHALACION, 1 inhalador de 100 dosis</t>
+        </is>
+      </c>
+      <c r="D365" s="12" t="inlineStr">
+        <is>
+          <t>650967</t>
+        </is>
+      </c>
+      <c r="E365" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA EASYHALER 400 microgramos POLVO PARA INHALACION, 1 inhalador de 100 dosis</t>
+        </is>
+      </c>
+      <c r="F365" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G365" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H365" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I365" s="12" t="inlineStr">
+        <is>
+          <t>&lt;50 l/m</t>
+        </is>
+      </c>
+      <c r="J365" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K365" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11817</t>
+        </is>
+      </c>
+      <c r="L365" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M365" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=66671</t>
+        </is>
+      </c>
+      <c r="N365" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O365" s="12" t="inlineStr"/>
+      <c r="P365" s="12" t="inlineStr"/>
+    </row>
+    <row r="366" ht="40" customHeight="1">
+      <c r="A366" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B366" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C366" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA PULMICTAN INFANTIL 50 microgramos/INHALACION SUSPENSION PARA INHALACION EN ENVASE A PRESION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D366" s="12" t="inlineStr">
+        <is>
+          <t>656614</t>
+        </is>
+      </c>
+      <c r="E366" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA PULMICTAN INFANTIL 50 microgramos/INHALACION SUSPENSION PARA INHALACION EN ENVASE A PRESION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F366" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G366" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H366" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I366" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J366" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K366" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L366" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M366" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=59036</t>
+        </is>
+      </c>
+      <c r="N366" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O366" s="12" t="inlineStr"/>
+      <c r="P366" s="12" t="inlineStr"/>
+    </row>
+    <row r="367" ht="40" customHeight="1">
+      <c r="A367" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B367" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C367" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA PULMICTAN 200 microgramos/INHALACION SUSPENSION PARA INHALACION EN ENVASE A PRESION , 1 inhalador de 100 dosis</t>
+        </is>
+      </c>
+      <c r="D367" s="12" t="inlineStr">
+        <is>
+          <t>656615</t>
+        </is>
+      </c>
+      <c r="E367" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA PULMICTAN 200 microgramos/INHALACION SUSPENSION PARA INHALACION EN ENVASE A PRESION , 1 inhalador de 100 dosis</t>
+        </is>
+      </c>
+      <c r="F367" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G367" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H367" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I367" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J367" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K367" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L367" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M367" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=59035</t>
+        </is>
+      </c>
+      <c r="N367" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O367" s="12" t="inlineStr"/>
+      <c r="P367" s="12" t="inlineStr"/>
+    </row>
+    <row r="368" ht="40" customHeight="1">
+      <c r="A368" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B368" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C368" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA PULMICTAN 200 microgramos/INHALACION SUSPENSION PARA INHALACION EN ENVASE A PRESION , 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D368" s="12" t="inlineStr">
+        <is>
+          <t>686770</t>
+        </is>
+      </c>
+      <c r="E368" s="12" t="inlineStr">
+        <is>
+          <t>BUDESONIDA PULMICTAN 200 microgramos/INHALACION SUSPENSION PARA INHALACION EN ENVASE A PRESION , 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F368" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G368" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H368" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I368" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J368" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K368" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L368" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M368" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=59035</t>
+        </is>
+      </c>
+      <c r="N368" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O368" s="12" t="inlineStr"/>
+      <c r="P368" s="12" t="inlineStr"/>
+    </row>
+    <row r="369" ht="40" customHeight="1">
+      <c r="A369" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B369" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C369" s="12" t="inlineStr">
+        <is>
+          <t>NOVOPULM NOVOLIZER 200 microgramos POLVO PARA INHALACION , 1 inhalador + 1 cartucho de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D369" s="12" t="inlineStr">
+        <is>
+          <t>945436</t>
+        </is>
+      </c>
+      <c r="E369" s="12" t="inlineStr">
+        <is>
+          <t>NOVOPULM NOVOLIZER 200 microgramos POLVO PARA INHALACION , 1 inhalador + 1 cartucho de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F369" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G369" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H369" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I369" s="12" t="inlineStr">
+        <is>
+          <t>60-90 l/m</t>
+        </is>
+      </c>
+      <c r="J369" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K369" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11882</t>
+        </is>
+      </c>
+      <c r="L369" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M369" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=65536</t>
+        </is>
+      </c>
+      <c r="N369" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O369" s="12" t="inlineStr"/>
+      <c r="P369" s="12" t="inlineStr"/>
+    </row>
+    <row r="370" ht="40" customHeight="1">
+      <c r="A370" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B370" s="12" t="inlineStr">
+        <is>
+          <t>budesonida</t>
+        </is>
+      </c>
+      <c r="C370" s="12" t="inlineStr">
+        <is>
+          <t>NOVOPULM NOVOLIZER 400 microgramos POLVO PARA INHALACION , 1 inhalador + 1 cartucho de 100 dosis</t>
+        </is>
+      </c>
+      <c r="D370" s="12" t="inlineStr">
+        <is>
+          <t>652283</t>
+        </is>
+      </c>
+      <c r="E370" s="12" t="inlineStr">
+        <is>
+          <t>NOVOPULM NOVOLIZER 400 microgramos POLVO PARA INHALACION , 1 inhalador + 1 cartucho de 100 dosis</t>
+        </is>
+      </c>
+      <c r="F370" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 200-400 µg/12h
+D.màx: 800 µg/12h
+Asma baixa: 200-400 µg/24h
+Asma mitjana: 401-800 µg/24h
+Asma alta: 801-1.600 µg/24h</t>
+        </is>
+      </c>
+      <c r="G370" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H370" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I370" s="12" t="inlineStr">
+        <is>
+          <t>60-90 l/m</t>
+        </is>
+      </c>
+      <c r="J370" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K370" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11882</t>
+        </is>
+      </c>
+      <c r="L370" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M370" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=67103</t>
+        </is>
+      </c>
+      <c r="N370" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O370" s="12" t="inlineStr"/>
+      <c r="P370" s="12" t="inlineStr"/>
+    </row>
+    <row r="371" ht="40" customHeight="1">
+      <c r="A371" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B371" s="12" t="inlineStr">
+        <is>
+          <t>beclometasona</t>
+        </is>
+      </c>
+      <c r="C371" s="12" t="inlineStr">
+        <is>
+          <t>BECLO-ASMA 100 MICROGRAMOS/PULSACION SOLUCION PARA INHALACION EN ENVASE A PRESION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D371" s="12" t="inlineStr">
+        <is>
+          <t>714479</t>
+        </is>
+      </c>
+      <c r="E371" s="12" t="inlineStr">
+        <is>
+          <t>BECLO-ASMA 100 MICROGRAMOS/PULSACION SOLUCION PARA INHALACION EN ENVASE A PRESION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F371" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 250-500 µg/12h
+D.màx: 1.000 µg/12h
+Asma baixa: 200-500 µg/24h
+Asma mitjana: 501-1.000 µg/24h
+Asma alta: 1.001-2.000 µg/24h</t>
+        </is>
+      </c>
+      <c r="G371" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H371" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I371" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J371" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K371" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L371" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M371" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=81684</t>
+        </is>
+      </c>
+      <c r="N371" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O371" s="12" t="inlineStr"/>
+      <c r="P371" s="12" t="inlineStr"/>
+    </row>
+    <row r="372" ht="40" customHeight="1">
+      <c r="A372" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B372" s="12" t="inlineStr">
+        <is>
+          <t>beclometasona</t>
+        </is>
+      </c>
+      <c r="C372" s="12" t="inlineStr">
+        <is>
+          <t>BECLO-ASMA 50 MICROGRAMOS/PULSACION SOLUCION PARA INHALACION EN ENVASE A PRESION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="D372" s="12" t="inlineStr">
+        <is>
+          <t>714441</t>
+        </is>
+      </c>
+      <c r="E372" s="12" t="inlineStr">
+        <is>
+          <t>BECLO-ASMA 50 MICROGRAMOS/PULSACION SOLUCION PARA INHALACION EN ENVASE A PRESION, 1 inhalador de 200 dosis</t>
+        </is>
+      </c>
+      <c r="F372" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 250-500 µg/12h
+D.màx: 1.000 µg/12h
+Asma baixa: 200-500 µg/24h
+Asma mitjana: 501-1.000 µg/24h
+Asma alta: 1.001-2.000 µg/24h</t>
+        </is>
+      </c>
+      <c r="G372" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H372" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I372" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J372" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K372" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L372" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M372" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=81667</t>
+        </is>
+      </c>
+      <c r="N372" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O372" s="12" t="inlineStr"/>
+      <c r="P372" s="12" t="inlineStr"/>
+    </row>
+    <row r="373" ht="40" customHeight="1">
+      <c r="A373" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B373" s="12" t="inlineStr">
+        <is>
+          <t>mometasona</t>
+        </is>
+      </c>
+      <c r="C373" s="12" t="inlineStr">
+        <is>
+          <t>ASMANEX TWISTHALER 200 microgramos POLVO PARA INHALACION , 1 inhalador de 60 dosis</t>
+        </is>
+      </c>
+      <c r="D373" s="12" t="inlineStr">
+        <is>
+          <t>744516</t>
+        </is>
+      </c>
+      <c r="E373" s="12" t="inlineStr">
+        <is>
+          <t>ASMANEX TWISTHALER 200 microgramos POLVO PARA INHALACION , 1 inhalador de 60 dosis</t>
+        </is>
+      </c>
+      <c r="F373" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 136/150/50 µg/24h
+D.màx: 136/150/50 µg/24h
+Asma baixa: 200 µg/24h
+Asma mitjana: 400 µg/24h
+Asma alta: 800 µg/24h</t>
+        </is>
+      </c>
+      <c r="G373" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H373" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I373" s="12" t="inlineStr">
+        <is>
+          <t>&lt;50 l/m</t>
+        </is>
+      </c>
+      <c r="J373" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K373" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11894</t>
+        </is>
+      </c>
+      <c r="L373" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M373" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=65226</t>
+        </is>
+      </c>
+      <c r="N373" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O373" s="12" t="inlineStr"/>
+      <c r="P373" s="12" t="inlineStr">
+        <is>
+          <t>MATMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="374" ht="40" customHeight="1">
+      <c r="A374" s="12" t="inlineStr">
+        <is>
+          <t>GCI</t>
+        </is>
+      </c>
+      <c r="B374" s="12" t="inlineStr">
+        <is>
+          <t>mometasona</t>
+        </is>
+      </c>
+      <c r="C374" s="12" t="inlineStr">
+        <is>
+          <t>ASMANEX TWISTHALER 400 microgramos POLVO PARA INHALACION, 1 inhalador de 60 dosis</t>
+        </is>
+      </c>
+      <c r="D374" s="12" t="inlineStr">
+        <is>
+          <t>751271</t>
+        </is>
+      </c>
+      <c r="E374" s="12" t="inlineStr">
+        <is>
+          <t>ASMANEX TWISTHALER 400 microgramos POLVO PARA INHALACION, 1 inhalador de 60 dosis</t>
+        </is>
+      </c>
+      <c r="F374" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 136/150/50 µg/24h
+D.màx: 136/150/50 µg/24h
+Asma baixa: 200 µg/24h
+Asma mitjana: 400 µg/24h
+Asma alta: 800 µg/24h</t>
+        </is>
+      </c>
+      <c r="G374" s="12" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H374" s="12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I374" s="12" t="inlineStr">
+        <is>
+          <t>&lt;50 l/m</t>
+        </is>
+      </c>
+      <c r="J374" s="12" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K374" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11894</t>
+        </is>
+      </c>
+      <c r="L374" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M374" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=65236</t>
+        </is>
+      </c>
+      <c r="N374" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O374" s="12" t="inlineStr"/>
+      <c r="P374" s="12" t="inlineStr">
+        <is>
+          <t>MATMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="375" ht="40" customHeight="1">
+      <c r="A375" s="12" t="inlineStr">
+        <is>
+          <t>PENDENT</t>
+        </is>
+      </c>
+      <c r="B375" s="12" t="inlineStr">
+        <is>
+          <t>mometasona</t>
+        </is>
+      </c>
+      <c r="C375" s="12" t="inlineStr">
+        <is>
+          <t>MOMETASONA SANDOZ 50 MICROGRAMOS/DOSIS SUSPENSION PARA PULVERIZACION NASAL , 1 envase de 18 g (140 nebulizaciones)</t>
+        </is>
+      </c>
+      <c r="D375" s="12" t="inlineStr">
+        <is>
+          <t>695268</t>
+        </is>
+      </c>
+      <c r="E375" s="12" t="inlineStr">
+        <is>
+          <t>MOMETASONA SANDOZ 50 MICROGRAMOS/DOSIS SUSPENSION PARA PULVERIZACION NASAL , 1 envase de 18 g (140 nebulizaciones)</t>
+        </is>
+      </c>
+      <c r="F375" s="12" t="inlineStr">
+        <is>
+          <t>MPOC: 136/150/50 µg/24h
+D.màx: 136/150/50 µg/24h
+Asma baixa: 200 µg/24h
+Asma mitjana: 400 µg/24h
+Asma alta: 800 µg/24h</t>
+        </is>
+      </c>
+      <c r="G375" s="12" t="inlineStr">
+        <is>
+          <t>ICP</t>
+        </is>
+      </c>
+      <c r="H375" s="12" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="I375" s="12" t="inlineStr">
+        <is>
+          <t>20-30 l/m</t>
+        </is>
+      </c>
+      <c r="J375" s="12" t="inlineStr">
+        <is>
+          <t>Lenta</t>
+        </is>
+      </c>
+      <c r="K375" s="12" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11880</t>
+        </is>
+      </c>
+      <c r="L375" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M375" s="12" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=76859</t>
+        </is>
+      </c>
+      <c r="N375" s="12" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O375" s="12" t="inlineStr"/>
+      <c r="P375" s="12" t="inlineStr">
+        <is>
+          <t>MATMA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:P97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Novetats CIMA: 1 nous farmacos pendents de validacio
</commit_message>
<xml_diff>
--- a/inhaladors_MPOC_ASMA_Avanzado_FINAL.xlsx
+++ b/inhaladors_MPOC_ASMA_Avanzado_FINAL.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z179"/>
+  <dimension ref="A1:Z180"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="20.13" customWidth="1" style="28" min="1" max="1"/>
@@ -13112,6 +13112,81 @@
       </c>
       <c r="O179" s="29" t="inlineStr"/>
       <c r="P179" s="29" t="inlineStr"/>
+    </row>
+    <row r="180" ht="40" customHeight="1" s="28">
+      <c r="A180" s="29" t="inlineStr">
+        <is>
+          <t>LABA/LAMA</t>
+        </is>
+      </c>
+      <c r="B180" s="29" t="inlineStr">
+        <is>
+          <t>aclidinio + formoterol</t>
+        </is>
+      </c>
+      <c r="C180" s="29" t="inlineStr">
+        <is>
+          <t>BRIMICA GENUAIR 340 MICROGRAMOS/12 MICROGRAMOS POLVO PARA INHALACION, 60 dosis</t>
+        </is>
+      </c>
+      <c r="D180" s="29" t="inlineStr">
+        <is>
+          <t>770181</t>
+        </is>
+      </c>
+      <c r="E180" s="29" t="inlineStr">
+        <is>
+          <t>BRIMICA GENUAIR 340 MICROGRAMOS/12 MICROGRAMOS POLVO PARA INHALACION, 60 dosis</t>
+        </is>
+      </c>
+      <c r="F180" s="29" t="inlineStr">
+        <is>
+          <t>MPOC: 12/340 µg/12h
+D.màx: 12/340 µg/12h</t>
+        </is>
+      </c>
+      <c r="G180" s="29" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H180" s="29" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I180" s="29" t="inlineStr">
+        <is>
+          <t>60-90 l/m</t>
+        </is>
+      </c>
+      <c r="J180" s="29" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K180" s="29" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11878</t>
+        </is>
+      </c>
+      <c r="L180" s="29" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="M180" s="29" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=114963001IP</t>
+        </is>
+      </c>
+      <c r="N180" s="29" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O180" s="29" t="inlineStr"/>
+      <c r="P180" s="29" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="$A$1:$P$140"/>

</xml_diff>